<commit_message>
xlsx: retirer le rapport integral de l'onglet Synthese
L'onglet Synthese recopiait tout le rapport de synthese, ce qui portait le classeur a
46 Ko. L'outil d'envoi Gmail n'accepte les pieces jointes qu'en base64 inline et cette
taille depasse ce qu'un appel peut porter : la piece jointe partait tronquee sans erreur.
L'onglet ne garde plus que les statistiques et un renvoi vers le fichier .md, qui reste
la version complete du rapport.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GF7VjUV8G8etQY4Drri31
</commit_message>
<xml_diff>
--- a/outputs/humanup_market_mapping_2026-09-03.xlsx
+++ b/outputs/humanup_market_mapping_2026-09-03.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -611,1126 +611,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rapport de synthese</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t># Rapport de Synthèse — Market Mapping Humanup.io</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>**Date :** 2026-09-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>**Destinataires :** Valentin Murcia (Finance + Hospitality), Alexis (Industrie), Louis (Sales SaaS), Méroë Nguimbi (Sales général)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>## 1. Volumes par vertical</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>| Vertical | Destinataire | Lignes | Entreprises uniques | Contacts sourcés | % sourcé |</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>|---|---|---|---|---|---|</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>| Finance | Valentin | 38 / 40 | 18 | 5 | 13 % |</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>| Hospitality | Valentin | 40 / 40 | 19 | 3 | 8 % |</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>| Industrie | Alexis | 40 / 40 | 20 | 3 | 8 % |</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>| Sales SaaS | Louis | 40 / 40 | 20 | **20** | **50 %** |</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>| Sales général | Méroë | 40 / 40 | 20 | 3 | 8 % |</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>| **TOTAL** | | **198** | **97** | **34** | **17 %** |</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>**Répartition JOB / NEWS**</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>| Vertical | JOB | NEWS |</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>| Finance | 29 | 9 |</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>| Hospitality | 28 | 12 |</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>| Industrie | 28 | 12 |</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>| Sales SaaS | 28 | 12 |</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>| Sales général | 40 | 0 |</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>## 2. Top régions / villes / secteurs</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>**Finance** — Paris (75) domine avec 11 lignes, puis Lyon (69) 4, Douarnenez (29) 3, et une</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>diagonale francilienne périphérique (Orly 94, Le Blanc-Mesnil 93, Taverny 95). Secteurs : cabinets</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>d'expertise comptable indépendants en consolidation, ETI familiales industrielles, médico-social.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>**Hospitality** — Paris (75) très majoritaire (18 lignes), Chamonix (74) 4, puis un chapelet</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>d'établissements de province et d'outre-mer : Cognac (16), La Teste-de-Buch (33), Loir-et-Cher (41),</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Polynésie (987). Secteurs : hôtellerie 4-5* indépendante, ouvertures et pré-ouvertures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>**Industrie** — La verticale la plus régionale, conformément à la consigne géographique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Pays de la Loire en tête : Maine-et-Loire (49) 6 lignes, Vendée (85) 4. Puis Lot (46), Nord (59),</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Haute-Loire (43), Finistère (29). Secteurs : sous-traitance aéronautique, matériaux de construction,</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>électronique industrielle, agroalimentaire.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>**Sales SaaS** — Concentration parisienne assumée (75) 28 lignes, Lyon (69) 6, Hauts-de-Seine (92) 4,</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Yvelines (78) 2. Secteurs : SaaS vertical métier (santé au travail, expertise comptable, restauration),</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>deeptech, fintech B2B.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>**Sales général** — La mieux répartie : Marne (51) 4, Bouches-du-Rhône (13) 4, Haute-Garonne (31) 4,</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>puis Rhône (69), Tarn (81), Finistère (29). Secteurs : négoce de matériaux, instrumentation de mesure,</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>services à la personne, distribution B2B.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>## 3. Top 7 signaux business prioritaires</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>1. **MyUnisoft** (Saint-Quentin-en-Yvelines, 253 sal.) — Plan de 100 recrutements sur 2026, soit un</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   passage de 253 à 353 collaborateurs, sous actionnariat majoritaire **HgCapital**. Le meilleur signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   du jour : volume, capital patient, éditeur peu médiatisé. → **LOUIS**</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>2. **padoa** (Paris) — **Thoma Bravo** prend le majoritaire via son fonds Europe de 1,8 Md€ ;</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Five Arrows et Kamet réinvestissent. Plan d'expansion DACH annoncé, donc recrutements commerciaux</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   à venir. → **LOUIS**</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>3. **Groupe Derrey** (Étival-Clairefontaine, 88, 600 sal.) — Campagne de 26 postes en CDI dans le</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Grand Est, dont plusieurs profils commerce ; annonce technico-commercial ouverte à Épinal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Négociant en matériaux indépendant, exactement notre cible. → **MÉROË**</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>4. **N2JSoft / N2F** (Lyon, 70 → 130 sal. en un an, &gt; 10 M€ de CA) — Recrute simultanément</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Sales Enablement Manager, RevOps Manager et SDR : refonte complète de la machine commerciale</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   d'un éditeur indépendant et discret. → **LOUIS**</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>5. **FDG Group** (Orly, 94, 630 sal., 117 M€ de CA) — Deux postes de contrôle de gestion ouverts en</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   parallèle (business partner opérationnel + corporate) : renforcement net et simultané de l'équipe</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   CDG, signal classique de structuration. → **VALENTIN**</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>6. **Chauvin Arnoux** (instrumentation de mesure, groupe familial indépendant, 430 sal., 57 M€) —</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Création d'un poste d'ingénieur technico-commercial itinérant sur la zone Toulouse : ouverture de</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   territoire, pas un remplacement. → **MÉROË**</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>7. **Techmo Hygiène** (Le Blanc-Mesnil, 93, 280 sal., groupe familial indépendant depuis 1947) —</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Comptable général expérimenté avec encadrement de deux comptables fournisseurs : structuration de</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   la fonction comptable dans une PME patrimoniale. → **VALENTIN**</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>## 4. Récurrences</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Périmètre scanné : **172 entreprises** déjà ciblées par les fichiers des 01/09, 02/09 et 03/09.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Ces entreprises sont exclues de la nouvelle recherche, mais vérifiées pour signal frais (27/08 → 03/09).</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>**3 récurrences confirmées :**</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>- **Figeac Aéro** (aéronautique / défense) — Chiffre d'affaires T1 2026/27 à 111,8 M€, 21e trimestre</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  consécutif de croissance (+11,6 % organique), carnet de commandes record à 5 Md€ — 02/09/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  → Signal de croissance soutenue, angle Industrie et Finance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>- **Voyageurs du Monde** (tourisme sur mesure) — AVANTAGE (86,59 % du capital) annonce une offre</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  publique de retrait à 180 € par action et la sortie de cote d'Euronext Paris — 01/09/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  → Sortie de cote : réorganisation probable des fonctions support, angle Finance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>- **STIF** (industrie, sécurité explosion et stockage d'énergie) — Déclaration mensuelle de droits de</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  vote au 31/08 — 02/09/2026. Signal réglementaire de routine, **faible valeur commerciale**.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Le détail, y compris les pistes écartées faute de datation dans la fenêtre, est dans</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>`outputs/_recurrences_2026-09-03.md`.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>## 5. Filtres appliqués</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>**Liste noire** — appliquée aux cinq verticales : Big 4, next tier (Mazars, Grant Thornton, BDO, RSM,</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Baker Tilly), réseaux d'expertise comptable (In Extenso, Fiducial, Cerfrance, Exco, Sofarec),</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>scale-ups surmédiatisées, CAC 40, et cabinets d'intérim masquant le client final.</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>**Plafond 2000 salariés au niveau groupe** — exclusions prononcées aujourd'hui :</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Padam Mobility (filiale Siemens Mobility), Mabéo Industries (groupe Martin Belaysoud),</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Fnac Darty, Primagaz, Jacquet Brossard, Agicap (FT120, trop visible).</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Intermédiaires écartés pour employeur final masqué : Dream Catcher Sales, Tomcat Talents, Jobglober.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>Écartés faute d'effectif vérifiable : Nopillo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>**Alternance / stage** — zéro annonce en alternance, apprentissage, contrat pro ou stage dans les</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>fichiers livrés. Wimi a été écarté à ce titre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>**Anti-doublons 14 jours** — les 172 entreprises déjà ciblées sont absentes des cinq fichiers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>## 6. Dédoublonnage Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Le fichier de Méroë a été confronté au fichier de Louis sur la colonne `entreprise` :</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>**aucune entreprise retirée**, les deux agents ayant travaillé sur des périmètres disjoints</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>(l'agent Sales général avait pour consigne d'éviter les éditeurs SaaS et tech B2B).</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>Les deux fichiers sortent donc à 40 lignes pleines, 20 entreprises chacun, sans recouvrement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>## 7. Limites du run — à lire</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>Ce run mérite trois réserves explicites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>**Contacts non sourcés.** Sur 198 lignes, 34 seulement portent un nom. Le budget de recherche web de</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>la session (200 requêtes, partagé entre tous les agents) a été épuisé avant la phase de sourcing</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>nominatif sur quatre verticales sur cinq. Seul le fichier Sales SaaS de Louis atteint 50 % de contacts</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>nommés. **Aucun nom n'a été inventé** : les lignes non sourcées portent le tag `CONTACT_NON_SOURCE`</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>et des colonnes `nom` / `prenom` / `linkedin` vides, à enrichir via FullEnrich ou une session dédiée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>**Dates de publication majoritairement en `NC`.** Le proxy de cet environnement bloque en accès direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>la quasi-totalité des sources utiles — APEC, Indeed, Hellowork, LinkedIn, Welcome to the Jungle,</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>France Travail, Pappers, Societe.com, ainsi que la plupart des sites carrière. Le travail s'est fait</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>sur les extraits de résultats de recherche. Les annonces retenues sont des offres réellement en ligne</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>au 03/09/2026 à employeur nommé, mais la fenêtre « publiée dans les 7 derniers jours » n'est pas</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>confirmable pour la majorité d'entre elles. Chaque ligne porte sa date réelle ou `NC` dans les notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>**Deux écarts de volume assumés.** Finance sort à 38 lignes au lieu de 40 (la partie A, comptabilité</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>générale et contrôle de gestion, n'a pas trouvé une cinquième opportunité vérifiable). Sales général</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>sort à 40 lignes mais avec 40 JOB et 0 NEWS : toutes les pistes NEWS remontées ont été écartées après</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>vérification — dates réelles hors fenêtre (Partedis, FATEC Group, Aditec) ou effectif groupe au-dessus</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>du plafond. Aucun signal n'a été fabriqué pour combler le quota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>## 8. Fichiers livrés</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr"/>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>| Fichier | Lignes | Destinataire |</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>|---|---|---|</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>| `outputs/finance_2026-09-03.csv` | 38 | Valentin Murcia |</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>| `outputs/hospitality_2026-09-03.csv` | 40 | Valentin Murcia |</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>| `outputs/industrie_2026-09-03.csv` | 40 | Alexis |</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>| `outputs/sales_saas_2026-09-03.csv` | 40 | Louis |</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>| `outputs/sales_2026-09-03.csv` | 40 | Méroë Nguimbi |</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>| `outputs/humanup_market_mapping_2026-09-03.xlsx` | 6 onglets | Méroë Nguimbi |</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>| `outputs/rapport_synthese_2026-09-03.md` | — | Méroë Nguimbi |</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr"/>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>Fichiers intermédiaires conservés pour traçabilité : `_fin_a`, `_fin_a_complement`, `_fin_b`,</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>`_fin_c`, `_sales_complement`, `_recurrences`.</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr"/>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr"/>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>## 9. Actions prioritaires</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr"/>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>1. **Attaquer MyUnisoft et padoa aujourd'hui** (Louis). Ce sont les deux signaux les plus chauds du</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   jour et les seuls adossés à un fonds avec un plan de recrutement explicite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>2. **Lancer l'enrichissement FullEnrich** sur les 164 lignes `CONTACT_NON_SOURCE` avant toute</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   séquence d'approche : les fichiers Finance, Hospitality, Industrie et Sales général sont</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   inexploitables en l'état sans noms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>3. **Groupe Derrey** (Méroë) : 26 postes ouverts d'un coup chez un négociant indépendant de 600</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   salariés, c'est un mandat multi-postes potentiel, pas une mission unitaire.</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>4. **Requalifier les dates** des annonces marquées `NC` avant approche, depuis un poste ayant accès</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   à l'APEC et à LinkedIn : une annonce de plus de trois semaines change l'angle d'appel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>5. **Prévoir une session de sourcing dédiée** avec budget de recherche réservé, pour ne pas</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   reproduire l'épuisement constaté sur ce run.</t>
+          <t>Rapport de synthese complet : outputs/rapport_synthese_2026-09-03.md</t>
         </is>
       </c>
     </row>

</xml_diff>